<commit_message>
fix(docs): update Excel for operator invitation flow
- 06_API一覧: 運営スタッフ追加→招待、OperatorCreateRequest→OperatorInviteRequest
- 07_画面一覧: 運営スタッフ管理 description更新
- Aligns Excel SoT with openapi_admin.yaml invite flow changes (98a3ea8)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/adapt_基本設計_最終版.xlsx
+++ b/docs/design/adapt_基本設計_最終版.xlsx
@@ -38311,7 +38311,7 @@
       </c>
       <c r="E82" s="52" t="inlineStr">
         <is>
-          <t>運営スタッフ追加</t>
+          <t>運営スタッフ招待</t>
         </is>
       </c>
       <c r="F82" s="52" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="I82" s="52" t="inlineStr">
         <is>
-          <t>OperatorCreateRequest</t>
+          <t>OperatorInviteRequest</t>
         </is>
       </c>
       <c r="J82" s="52" t="inlineStr">
@@ -38351,7 +38351,7 @@
       </c>
       <c r="M82" s="52" t="inlineStr">
         <is>
-          <t>既存ユーザーのglobalRoleをoperator/root_operatorに変更し運営スタッフとして登録。</t>
+          <t>メールアドレスで運営スタッフを招待。Keycloakにユーザーを作成しパスワード設定リンク付き招待メールを送信。globalRoleをoperator/root_operatorに設定。learner/instructorからの昇格ではなく、新規の運営スタッフ専用アカウントを作成する。招待メール送信元はTBD。</t>
         </is>
       </c>
     </row>
@@ -40168,7 +40168,7 @@
       </c>
       <c r="E46" s="36" t="inlineStr">
         <is>
-          <t>運営スタッフ管理</t>
+          <t>メール招待による運営スタッフ追加。root_operatorがメールアドレスと付与ロール(operator/root_operator)を指定して招待メールを送信。招待されたユーザーはauth.adapt-co.io(Keycloak)でアカウント作成・パスワード設定を行いログイン可能となる。learner/instructorからの昇格ではない。</t>
         </is>
       </c>
       <c r="F46" s="17" t="inlineStr">

</xml_diff>

<commit_message>
docs: openapi_app.yaml API-043/045 レスポンス型を一覧型に変更（SubmissionListResponse/CourseMemberListResponse追加）
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/design/adapt_基本設計_最終版.xlsx
+++ b/docs/design/adapt_基本設計_最終版.xlsx
@@ -36088,7 +36088,7 @@
       </c>
       <c r="J44" s="45" t="inlineStr">
         <is>
-          <t>CourseDetailView</t>
+          <t>SubmissionListResponse</t>
         </is>
       </c>
       <c r="K44" s="45" t="inlineStr">
@@ -36218,7 +36218,7 @@
       </c>
       <c r="J46" s="45" t="inlineStr">
         <is>
-          <t>CourseDetailView</t>
+          <t>CourseMemberListResponse</t>
         </is>
       </c>
       <c r="K46" s="45" t="inlineStr">

</xml_diff>